<commit_message>
test: validate login with locked out user
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>CT</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t>002</t>
+  </si>
+  <si>
+    <t>locked_out_user</t>
   </si>
   <si>
     <t>003</t>
@@ -387,7 +390,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="20.13"/>
+    <col customWidth="1" min="2" max="2" width="23.0"/>
     <col customWidth="1" min="3" max="3" width="21.63"/>
     <col customWidth="1" min="4" max="4" width="31.38"/>
     <col customWidth="1" min="5" max="5" width="18.38"/>
@@ -485,8 +488,12 @@
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+      <c r="B3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -509,13 +516,13 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -539,7 +546,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -565,7 +572,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -591,7 +598,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -617,7 +624,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -643,7 +650,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -669,7 +676,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -695,7 +702,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -721,7 +728,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -747,7 +754,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -773,7 +780,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -799,7 +806,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -825,7 +832,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>

</xml_diff>

<commit_message>
test: validate login without credentials
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>CT</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>003</t>
-  </si>
-  <si>
-    <t>TESTE</t>
   </si>
   <si>
     <t>004</t>
@@ -518,12 +515,8 @@
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -546,7 +539,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -572,7 +565,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -598,7 +591,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -624,7 +617,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -650,7 +643,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -676,7 +669,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -702,7 +695,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -728,7 +721,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -754,7 +747,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -780,7 +773,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -806,7 +799,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -832,7 +825,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>

</xml_diff>

<commit_message>
test: validate remove product from cart
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="29">
   <si>
     <t>CT</t>
   </si>
@@ -76,10 +76,13 @@
     <t>009</t>
   </si>
   <si>
-    <t>Backpack</t>
+    <t>Sauce Labs Backpack</t>
   </si>
   <si>
     <t>010</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bolt T-Shirt</t>
   </si>
   <si>
     <t>011</t>
@@ -378,7 +381,7 @@
     <col customWidth="1" min="2" max="2" width="23.0"/>
     <col customWidth="1" min="3" max="3" width="21.63"/>
     <col customWidth="1" min="4" max="4" width="31.88"/>
-    <col customWidth="1" min="5" max="5" width="27.13"/>
+    <col customWidth="1" min="5" max="5" width="30.63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,10 +608,16 @@
       <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+      <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="E11" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -620,10 +629,14 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="B12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="4"/>
@@ -637,10 +650,14 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="B13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="4"/>
@@ -654,10 +671,14 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="B14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="4"/>
@@ -671,10 +692,14 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="B15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="4"/>
@@ -688,10 +713,14 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="B16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="4"/>

</xml_diff>

<commit_message>
test: continue shopping after adding product to cart
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="29">
   <si>
     <t>CT</t>
   </si>
@@ -638,7 +638,9 @@
         <v>7</v>
       </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="E12" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>

</xml_diff>

<commit_message>
test: validate checkout information submission
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="34">
   <si>
     <t>CT</t>
   </si>
@@ -26,6 +26,15 @@
   </si>
   <si>
     <t>PRODUCT</t>
+  </si>
+  <si>
+    <t>FIRST_NAME</t>
+  </si>
+  <si>
+    <t>LAST_NAME</t>
+  </si>
+  <si>
+    <t>ZIP_CODE</t>
   </si>
   <si>
     <t>001</t>
@@ -89,6 +98,12 @@
   </si>
   <si>
     <t>012</t>
+  </si>
+  <si>
+    <t>TESTE</t>
+  </si>
+  <si>
+    <t>ASDF</t>
   </si>
   <si>
     <t>013</t>
@@ -382,6 +397,9 @@
     <col customWidth="1" min="3" max="3" width="21.63"/>
     <col customWidth="1" min="4" max="4" width="31.88"/>
     <col customWidth="1" min="5" max="5" width="30.63"/>
+    <col customWidth="1" min="6" max="6" width="20.0"/>
+    <col customWidth="1" min="7" max="7" width="18.88"/>
+    <col customWidth="1" min="8" max="8" width="16.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -400,9 +418,15 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
@@ -411,19 +435,19 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -432,19 +456,19 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -453,15 +477,15 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -470,19 +494,19 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -491,21 +515,21 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E6" s="1"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -514,21 +538,21 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -537,21 +561,21 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
@@ -560,21 +584,21 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E9" s="1"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
@@ -583,21 +607,21 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -606,21 +630,21 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
@@ -629,21 +653,21 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
@@ -652,19 +676,27 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
+      <c r="E13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="2">
+        <v>12345.0</v>
+      </c>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -673,19 +705,19 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -694,19 +726,19 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -715,19 +747,19 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>

</xml_diff>

<commit_message>
test: validate error message on checkout page
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
   <si>
     <t>CT</t>
   </si>
@@ -714,7 +714,9 @@
         <v>10</v>
       </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="E14" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>

</xml_diff>

<commit_message>
test: validate item added to cart on checkout overview page
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="34">
   <si>
     <t>CT</t>
   </si>
@@ -737,10 +737,18 @@
         <v>10</v>
       </c>
       <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="E15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" s="2">
+        <v>12345.0</v>
+      </c>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -758,7 +766,9 @@
         <v>10</v>
       </c>
       <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+      <c r="E16" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>

</xml_diff>